<commit_message>
Scores added to dataframe and saved to xlsx
</commit_message>
<xml_diff>
--- a/Odds-Data-Clean/2019-20.xlsx
+++ b/Odds-Data-Clean/2019-20.xlsx
@@ -419,12 +419,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -461,12 +461,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -503,12 +503,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -545,12 +545,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -587,12 +587,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -629,12 +629,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -671,12 +671,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -711,14 +711,10 @@
           <t>2019-20-1023</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -755,12 +751,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -797,12 +793,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -839,14 +835,10 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Utah</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+          <t>Utah Jazz</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
         <v>222</v>
       </c>
@@ -881,12 +873,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -923,12 +915,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -965,12 +957,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1007,12 +999,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1049,12 +1041,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1091,12 +1083,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1133,12 +1125,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1173,14 +1165,10 @@
           <t>2019-20-1025</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1215,14 +1203,10 @@
           <t>2019-20-1025</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1259,12 +1243,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1301,12 +1285,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1343,12 +1327,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1385,12 +1369,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1427,12 +1411,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1469,12 +1453,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1511,12 +1495,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1553,12 +1537,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1595,12 +1579,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1637,12 +1621,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -1679,12 +1663,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -1721,12 +1705,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -1763,12 +1747,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -1805,12 +1789,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -1847,12 +1831,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -1887,14 +1871,10 @@
           <t>2019-20-1027</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -1931,14 +1911,10 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Memphis</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+          <t>Memphis Grizzlies</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
         <v>224</v>
       </c>
@@ -1973,12 +1949,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -2015,12 +1991,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -2057,12 +2033,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -2099,12 +2075,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -2141,12 +2117,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -2183,12 +2159,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -2225,12 +2201,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -2267,12 +2243,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -2309,12 +2285,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -2351,14 +2327,10 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Houston</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+          <t>Houston Rockets</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
       <c r="E48" t="n">
         <v>225</v>
       </c>
@@ -2393,12 +2365,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -2435,12 +2407,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -2477,12 +2449,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -2519,12 +2491,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -2561,12 +2533,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -2603,12 +2575,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -2645,12 +2617,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -2687,12 +2659,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -2729,12 +2701,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -2771,12 +2743,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -2813,12 +2785,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -2853,14 +2825,10 @@
           <t>2019-20-1030</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -2897,12 +2865,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -2939,12 +2907,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -2979,14 +2947,10 @@
           <t>2019-20-1030</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -3023,12 +2987,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -3065,12 +3029,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -3107,12 +3071,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -3149,12 +3113,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -3191,12 +3155,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -3233,12 +3197,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -3273,14 +3237,10 @@
           <t>2019-20-1101</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -3317,12 +3277,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -3359,12 +3319,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -3401,12 +3361,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -3443,12 +3403,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -3485,12 +3445,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -3527,12 +3487,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -3569,12 +3529,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -3609,14 +3569,10 @@
           <t>2019-20-1102</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+      <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -3653,14 +3609,10 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Detroit</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+          <t>Detroit Pistons</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
       <c r="E79" t="n">
         <v>224</v>
       </c>
@@ -3695,12 +3647,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -3737,12 +3689,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -3779,12 +3731,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -3821,12 +3773,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -3863,12 +3815,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -3905,12 +3857,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -3947,12 +3899,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -3989,12 +3941,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -4031,12 +3983,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -4073,12 +4025,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -4115,12 +4067,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -4157,12 +4109,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -4199,12 +4151,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -4239,14 +4191,10 @@
           <t>2019-20-1104</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -4283,12 +4231,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -4325,12 +4273,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="E95" t="n">
@@ -4367,12 +4315,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="E96" t="n">
@@ -4409,12 +4357,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E97" t="n">
@@ -4451,12 +4399,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E98" t="n">
@@ -4493,12 +4441,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="E99" t="n">
@@ -4535,12 +4483,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E100" t="n">
@@ -4575,14 +4523,10 @@
           <t>2019-20-1105</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+      <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -4619,12 +4563,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -4661,12 +4605,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -4703,12 +4647,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -4745,12 +4689,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="E105" t="n">
@@ -4787,12 +4731,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="E106" t="n">
@@ -4829,12 +4773,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E107" t="n">
@@ -4871,12 +4815,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="E108" t="n">
@@ -4913,12 +4857,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="E109" t="n">
@@ -4955,12 +4899,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="E110" t="n">
@@ -4997,12 +4941,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="E111" t="n">
@@ -5039,12 +4983,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -5081,12 +5025,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -5123,14 +5067,10 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
       <c r="E114" t="n">
         <v>214.5</v>
       </c>
@@ -5165,12 +5105,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -5207,12 +5147,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -5249,12 +5189,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E117" t="n">
@@ -5291,12 +5231,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E118" t="n">
@@ -5333,12 +5273,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="E119" t="n">
@@ -5375,12 +5315,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -5417,12 +5357,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -5459,12 +5399,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="E122" t="n">
@@ -5501,12 +5441,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -5543,12 +5483,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -5585,12 +5525,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="E125" t="n">
@@ -5627,14 +5567,10 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Portland</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+          <t>Portland Trail Blazers</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
       <c r="E126" t="n">
         <v>233</v>
       </c>
@@ -5669,12 +5605,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -5711,12 +5647,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -5753,12 +5689,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -5793,14 +5729,10 @@
           <t>2019-20-1109</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+      <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -5837,12 +5769,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="E131" t="n">
@@ -5879,12 +5811,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -5921,12 +5853,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -5963,12 +5895,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -6005,12 +5937,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -6045,14 +5977,10 @@
           <t>2019-20-1110</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+      <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -6089,12 +6017,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -6131,14 +6059,10 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Phoenix</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+          <t>Phoenix Suns</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr"/>
       <c r="E138" t="n">
         <v>233</v>
       </c>
@@ -6173,12 +6097,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E139" t="n">
@@ -6215,12 +6139,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -6257,12 +6181,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="E141" t="n">
@@ -6299,12 +6223,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="E142" t="n">
@@ -6341,12 +6265,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="E143" t="n">
@@ -6383,12 +6307,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="E144" t="n">
@@ -6425,12 +6349,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="E145" t="n">
@@ -6467,12 +6391,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="E146" t="n">
@@ -6509,12 +6433,12 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E147" t="n">
@@ -6551,14 +6475,10 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Indiana</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+          <t>Indiana Pacers</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr"/>
       <c r="E148" t="n">
         <v>209.5</v>
       </c>
@@ -6593,12 +6513,12 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E149" t="n">
@@ -6635,12 +6555,12 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E150" t="n">
@@ -6677,12 +6597,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="E151" t="n">
@@ -6719,12 +6639,12 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E152" t="n">
@@ -6761,14 +6681,10 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Utah</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+          <t>Utah Jazz</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr"/>
       <c r="E153" t="n">
         <v>217</v>
       </c>
@@ -6803,12 +6719,12 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E154" t="n">
@@ -6845,12 +6761,12 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="E155" t="n">
@@ -6887,12 +6803,12 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -6929,12 +6845,12 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="E157" t="n">
@@ -6971,12 +6887,12 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="E158" t="n">
@@ -7013,12 +6929,12 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E159" t="n">
@@ -7055,12 +6971,12 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="E160" t="n">
@@ -7097,12 +7013,12 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E161" t="n">
@@ -7139,12 +7055,12 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="E162" t="n">
@@ -7181,12 +7097,12 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="E163" t="n">
@@ -7223,12 +7139,12 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="E164" t="n">
@@ -7265,12 +7181,12 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="E165" t="n">
@@ -7307,12 +7223,12 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E166" t="n">
@@ -7349,14 +7265,10 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Denver</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+          <t>Denver Nuggets</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr"/>
       <c r="E167" t="n">
         <v>225.5</v>
       </c>
@@ -7391,12 +7303,12 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E168" t="n">
@@ -7433,12 +7345,12 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E169" t="n">
@@ -7475,12 +7387,12 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="E170" t="n">
@@ -7517,12 +7429,12 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="E171" t="n">
@@ -7557,14 +7469,10 @@
           <t>2019-20-1115</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+      <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="E172" t="n">
@@ -7601,12 +7509,12 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="E173" t="n">
@@ -7643,12 +7551,12 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E174" t="n">
@@ -7685,12 +7593,12 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="E175" t="n">
@@ -7727,14 +7635,10 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Chicago</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+          <t>Chicago Bulls</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr"/>
       <c r="E176" t="n">
         <v>231.5</v>
       </c>
@@ -7769,12 +7673,12 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="E177" t="n">
@@ -7811,12 +7715,12 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="E178" t="n">
@@ -7853,12 +7757,12 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="E179" t="n">
@@ -7895,12 +7799,12 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E180" t="n">
@@ -7937,12 +7841,12 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="E181" t="n">
@@ -7979,12 +7883,12 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E182" t="n">
@@ -8021,12 +7925,12 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E183" t="n">
@@ -8063,12 +7967,12 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="E184" t="n">
@@ -8105,12 +8009,12 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E185" t="n">
@@ -8147,12 +8051,12 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="E186" t="n">
@@ -8189,12 +8093,12 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="E187" t="n">
@@ -8231,12 +8135,12 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E188" t="n">
@@ -8273,12 +8177,12 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E189" t="n">
@@ -8315,12 +8219,12 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E190" t="n">
@@ -8355,14 +8259,10 @@
           <t>2019-20-1118</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+      <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="E191" t="n">
@@ -8399,12 +8299,12 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="E192" t="n">
@@ -8441,12 +8341,12 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="E193" t="n">
@@ -8483,12 +8383,12 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E194" t="n">
@@ -8525,12 +8425,12 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E195" t="n">
@@ -8567,12 +8467,12 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="E196" t="n">
@@ -8609,12 +8509,12 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E197" t="n">
@@ -8651,14 +8551,10 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>LAClippers</t>
-        </is>
-      </c>
-      <c r="D198" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+          <t>Los Angeles Clippers</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr"/>
       <c r="E198" t="n">
         <v>219.5</v>
       </c>
@@ -8693,12 +8589,12 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E199" t="n">
@@ -8735,12 +8631,12 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E200" t="n">
@@ -8777,12 +8673,12 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="E201" t="n">
@@ -8819,14 +8715,10 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>LALakers</t>
-        </is>
-      </c>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr"/>
       <c r="E202" t="n">
         <v>210.5</v>
       </c>
@@ -8861,12 +8753,12 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>NewYork</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E203" t="n">
@@ -8903,12 +8795,12 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E204" t="n">
@@ -8945,12 +8837,12 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E205" t="n">
@@ -8987,12 +8879,12 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="E206" t="n">
@@ -9029,12 +8921,12 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E207" t="n">
@@ -9069,14 +8961,10 @@
           <t>2019-20-1120</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+      <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="E208" t="n">
@@ -9113,12 +9001,12 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="E209" t="n">
@@ -9155,12 +9043,12 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E210" t="n">
@@ -9197,12 +9085,12 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="E211" t="n">
@@ -9239,12 +9127,12 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="E212" t="n">
@@ -9281,12 +9169,12 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E213" t="n">
@@ -9323,12 +9211,12 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E214" t="n">
@@ -9365,12 +9253,12 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>NewOrleans</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E215" t="n">
@@ -9407,12 +9295,12 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E216" t="n">
@@ -9449,12 +9337,12 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Charlotte Bobcats</t>
         </is>
       </c>
       <c r="E217" t="n">
@@ -9489,14 +9377,10 @@
           <t>2019-20-1122</t>
         </is>
       </c>
-      <c r="C218" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+      <c r="C218" t="inlineStr"/>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="E218" t="n">
@@ -9533,12 +9417,12 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>SanAntonio</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E219" t="n">
@@ -9575,12 +9459,12 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="E220" t="n">
@@ -9615,14 +9499,10 @@
           <t>2019-20-1122</t>
         </is>
       </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>OklahomaCity</t>
-        </is>
-      </c>
+      <c r="C221" t="inlineStr"/>
       <c r="D221" t="inlineStr">
         <is>
-          <t>LALakers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="E221" t="n">
@@ -9659,12 +9539,12 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E222" t="n">
@@ -9701,12 +9581,12 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E223" t="n">
@@ -9743,12 +9623,12 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>GoldenState</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E224" t="n">
@@ -9785,12 +9665,12 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>LAClippers</t>
+          <t>Los Angeles Clippers</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="E225" t="n">

</xml_diff>